<commit_message>
Incorporar version final final del reparto de Ruge (editada por Mariano)
Mariano completo a mano los 49 items que habian quedado sin encargado
y resubio el excel por persona como version definitiva. Se sincroniza
con el maestro (Detalle completo por item, Resumen por bloque) y se
regenera ruge_reparto_lookup.md: 202/202 items con encargado, cero sin
asignar. Se corrige el nombre de un item (mantel verde, no negro, por
lo dicho en la llamada). ClickUp sigue con rate limit (confirmado de
nuevo, ~794 min restantes) - la sincronizacion queda para el
send_later ya programado.
</commit_message>
<xml_diff>
--- a/mariano-os/areas/ministerio/recursos/Ruge_reparto_tareas_17ago2026_actualizado.xlsx
+++ b/mariano-os/areas/ministerio/recursos/Ruge_reparto_tareas_17ago2026_actualizado.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="14">
     <font>
       <name val="Calibri"/>
@@ -187,7 +189,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -249,6 +251,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -673,7 +678,11 @@
           <t>26 ago</t>
         </is>
       </c>
-      <c r="F7" s="12" t="n"/>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>Ver detalle por ítem (repartido)</t>
+        </is>
+      </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
           <t>Ver miercoles 19 ago (pendiente respuesta de Mauricio sobre lote de piscina)</t>
@@ -686,7 +695,7 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>PENDIENTE 17 ago: parte de esto (arena, cajas de requisa, cuerdas de piscina) podria ser del equipo de Eventos (Mauricio y Cristian, lo gestionaron el reto pasado) - Julio le pregunta a Mauricio quien lo compro y donde antes de asignar encargado final. | ACTUALIZADO 17 ago (2da revision, tras subir el inventario real): se sumaron 26 items mas que figuraban como ALMACEN RUGE en el inventario original y se habian quedado afuera del detalle. Ninguno se discutio en la llamada, siguen sin encargado.</t>
+          <t>PENDIENTE 17 ago: parte de esto (arena, cajas de requisa, cuerdas de piscina) podria ser del equipo de Eventos (Mauricio y Cristian, lo gestionaron el reto pasado) - Julio le pregunta a Mauricio quien lo compro y donde antes de asignar encargado final. | ACTUALIZADO 17 ago (2da revision, tras subir el inventario real): se sumaron 26 items mas que figuraban como ALMACEN RUGE en el inventario original y se habian quedado afuera del detalle. Ninguno se discutio en la llamada, siguen sin encargado. | REPARTO FINAL 17 ago (version de Mariano, ver ruge_reparto_lookup.md): Repartido: David Luzuriaga (29 items), Marco Guanuchi (4 items) - version final de Mariano 17 ago.</t>
         </is>
       </c>
     </row>
@@ -851,7 +860,7 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Marco Guanuchi</t>
+          <t>Ver detalle por ítem (repartido)</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
@@ -866,7 +875,7 @@
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
-          <t>Pedir a Nestor si puede prestar nuevamente las cuerdas, Pedir estuche insulina a Marco,  mantel verde, las mesas ya están en Xodos, Pedir radios (y ver si funcionan todas a Administración de la iglesia), altavoz pedir a Chiriguaya | ACTUALIZADO 17 ago (llamada reparto): Altavoz: pedir a Chiriguaya. Cuerdas: pedirle a Nestor si las vuelve a prestar (las presto el la vez pasada). Estuche de insulina: lo tiene Marco Guanuchi. Mantel verde: comprar. Mesas: ya estan en Xodos, confirmar. Radios de iglesia x10: hablar con Juliana (administracion) y verificar que funcionen todas.</t>
+          <t>Pedir a Nestor si puede prestar nuevamente las cuerdas, Pedir estuche insulina a Marco,  mantel verde, las mesas ya están en Xodos, Pedir radios (y ver si funcionan todas a Administración de la iglesia), altavoz pedir a Chiriguaya | ACTUALIZADO 17 ago (llamada reparto): Altavoz: pedir a Chiriguaya. Cuerdas: pedirle a Nestor si las vuelve a prestar (las presto el la vez pasada). Estuche de insulina: lo tiene Marco Guanuchi. Mantel verde: comprar. Mesas: ya estan en Xodos, confirmar. Radios de iglesia x10: hablar con Juliana (administracion) y verificar que funcionen todas. | REPARTO FINAL 17 ago (version de Mariano, ver ruge_reparto_lookup.md): Mayoría Marco Guanuchi, 1 ítem (alargador eléctrico) con Julio Cesar Navia.</t>
         </is>
       </c>
     </row>
@@ -896,7 +905,7 @@
       </c>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>Julio Cesar Navia</t>
+          <t>Ver detalle por ítem (repartido)</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
@@ -911,7 +920,7 @@
       </c>
       <c r="I12" s="15" t="inlineStr">
         <is>
-          <t>Julio se hace cargo de hablar con Mateo y Jefferson por camion cerrado y furgoneta, Marco del bus y lo ve con Guanuchi, David de la pick up, Marco de radios y telefonos satalitales. Julio se encarga del conjunto de tareas | ACTUALIZADO 17 ago (llamada reparto): Bus 55 plazas: Marco Guanuchi habla con Andres Uquillas (quien lo alquilo la vez pasada) por el mismo presupuesto para la nueva fecha, Julio le hace seguimiento. Camion cerrado y furgoneta: Julio habla con Mateo y Jefferson. Radios VHF x15 y telefonos satelitales x2: Marco Guanuchi busca la empresa de alquiler. Troncos: Julio contacta al mismo vendedor con el que nego Marco Jurado el ano pasado, para el 2-3 de octubre. Pick-up / camion caja abierta: David busca donde alquilarla. Julio es el encargado del conjunto y le reporta a Mariano.</t>
+          <t>Julio se hace cargo de hablar con Mateo y Jefferson por camion cerrado y furgoneta, Marco del bus y lo ve con Guanuchi, David de la pick up, Marco de radios y telefonos satalitales. Julio se encarga del conjunto de tareas | ACTUALIZADO 17 ago (llamada reparto): Bus 55 plazas: Marco Guanuchi habla con Andres Uquillas (quien lo alquilo la vez pasada) por el mismo presupuesto para la nueva fecha, Julio le hace seguimiento. Camion cerrado y furgoneta: Julio habla con Mateo y Jefferson. Radios VHF x15 y telefonos satelitales x2: Marco Guanuchi busca la empresa de alquiler. Troncos: Julio contacta al mismo vendedor con el que nego Marco Jurado el ano pasado, para el 2-3 de octubre. Pick-up / camion caja abierta: David busca donde alquilarla. Julio es el encargado del conjunto y le reporta a Mariano. | REPARTO FINAL 17 ago (version de Mariano, ver ruge_reparto_lookup.md): Repartido: Marco Guanuchi (bus, radios VHF, satelital), Julio Cesar Navia (camión cerrado, furgoneta, troncos), David Luzuriaga (camión caja abierta).</t>
         </is>
       </c>
     </row>
@@ -941,7 +950,7 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Julio Cesar Navia</t>
+          <t>Ver detalle por ítem (repartido)</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
@@ -956,7 +965,7 @@
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
-          <t>Julio habla con Mauricio para saber quién compró todo y pide presupuestos, ,Marco se encarga de figuras de premios hablar con Richard, Fuegos pirotecnicos hablar con el pastor, guantes normales, paja donde se compra la arena, tierra es lo mismo. | ACTUALIZADO 17 ago (llamada reparto): Bolsas de basura y ziploc: Mercadona. Fuegos pirotecnicos y guantes normales: cualquier sitio (guantes ya acordados con Marco Jurado). Cinta reflectante y figuras de premios: van con el contacto de Marco Jurado / su sobrino Richard, dentro del bloque de Julio (Mariano NO gestiona esto directo — el solo recibe el presupuesto final para pasarlo a administracion, como coordinador general, no como ejecutor de tareas de campo). Arena y paja son del lote de piscina - Julio le pregunta a Mauricio (Eventos) quien lo compro y donde el reto pasado, pendiente su respuesta antes de asignar encargado final de esa parte.</t>
+          <t>Julio habla con Mauricio para saber quién compró todo y pide presupuestos, ,Marco se encarga de figuras de premios hablar con Richard, Fuegos pirotecnicos hablar con el pastor, guantes normales, paja donde se compra la arena, tierra es lo mismo. | ACTUALIZADO 17 ago (llamada reparto): Bolsas de basura y ziploc: Mercadona. Fuegos pirotecnicos y guantes normales: cualquier sitio (guantes ya acordados con Marco Jurado). Cinta reflectante y figuras de premios: van con el contacto de Marco Jurado / su sobrino Richard, dentro del bloque de Julio (Mariano NO gestiona esto directo — el solo recibe el presupuesto final para pasarlo a administracion, como coordinador general, no como ejecutor de tareas de campo). Arena y paja son del lote de piscina - Julio le pregunta a Mauricio (Eventos) quien lo compro y donde el reto pasado, pendiente su respuesta antes de asignar encargado final de esa parte. | REPARTO FINAL 17 ago (version de Mariano, ver ruge_reparto_lookup.md): Repartido: Marco Guanuchi (9), Julio Cesar Navia (7), David Luzuriaga (7) - version final de Mariano 17 ago.</t>
         </is>
       </c>
     </row>
@@ -2605,7 +2614,7 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Iglesia Impact Valencia</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
@@ -2641,7 +2650,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Prestado por Marcos J.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Prestado por Marcos J.</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
@@ -2678,8 +2687,16 @@
         <v>30</v>
       </c>
       <c r="F7" s="9" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="10" t="n"/>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
@@ -2704,8 +2721,16 @@
         <v>90</v>
       </c>
       <c r="F8" s="9" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
@@ -2730,8 +2755,16 @@
         <v>5</v>
       </c>
       <c r="F9" s="9" t="n"/>
-      <c r="G9" s="10" t="n"/>
-      <c r="H9" s="10" t="n"/>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
@@ -2756,8 +2789,16 @@
         <v>5</v>
       </c>
       <c r="F10" s="9" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
@@ -2781,9 +2822,19 @@
       <c r="E11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="10" t="n"/>
-      <c r="H11" s="10" t="n"/>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
@@ -2805,9 +2856,19 @@
       <c r="E12" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="10" t="n"/>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
@@ -2832,8 +2893,16 @@
         <v>200</v>
       </c>
       <c r="F13" s="9" t="n"/>
-      <c r="G13" s="10" t="n"/>
-      <c r="H13" s="10" t="n"/>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -2857,7 +2926,7 @@
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Metal o madera desmontable — valorar que la haga Néstor</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Metal o madera desmontable — valorar que la haga Néstor</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
@@ -2893,7 +2962,7 @@
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Mandarlo hacer — Levis</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Mandarlo hacer — Levis</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
@@ -2929,7 +2998,7 @@
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Mandarlo hacer — Levis</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Mandarlo hacer — Levis</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
@@ -2965,7 +3034,7 @@
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Mandarlo hacer — Marcos Chiriguaya</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Mandarlo hacer — Marcos Chiriguaya</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
@@ -3065,7 +3134,7 @@
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Necesita tiempo de envío desde Costa Rica</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
@@ -3101,7 +3170,7 @@
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Sumar talla doble de grande (corrección retrospectiva)</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
@@ -3135,7 +3204,11 @@
       <c r="E22" s="9" t="n">
         <v>50</v>
       </c>
-      <c r="F22" s="9" t="n"/>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
+        </is>
+      </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
           <t>Marco Guanuchi</t>
@@ -3169,7 +3242,7 @@
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Por comisión</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
@@ -3205,7 +3278,7 @@
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Sumar talla doble de grande (corrección retrospectiva)</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
@@ -3239,7 +3312,11 @@
       <c r="E25" s="9" t="n">
         <v>60</v>
       </c>
-      <c r="F25" s="9" t="n"/>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
+        </is>
+      </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
           <t>Marco Guanuchi</t>
@@ -3273,7 +3350,7 @@
       </c>
       <c r="F26" s="9" t="inlineStr">
         <is>
-          <t>Marcos Chiriguaya y Mariano B.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Marcos Chiriguaya y Mariano B.</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
@@ -3309,7 +3386,7 @@
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Néstor</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Néstor</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
@@ -3347,7 +3424,7 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>Marco Guanuchi</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Marco Guanuchi</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
@@ -3374,7 +3451,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>MANTEL NEGRO PARA MESA DE CAMISETAS</t>
+          <t>MANTEL VERDE PARA MESA DE CAMISETAS</t>
         </is>
       </c>
       <c r="D29" s="9" t="n"/>
@@ -3383,7 +3460,7 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>Iglesia Impact Valencia</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
@@ -3419,7 +3496,7 @@
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
-          <t>Local multiusos Xodos</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Local multiusos Xodos</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
@@ -3455,7 +3532,7 @@
       </c>
       <c r="F31" s="9" t="inlineStr">
         <is>
-          <t>Iglesia Impact Valencia</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
         </is>
       </c>
       <c r="G31" s="10" t="inlineStr">
@@ -3491,7 +3568,7 @@
       </c>
       <c r="F32" s="9" t="inlineStr">
         <is>
-          <t>Algún servidor</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Buscar alquiler y pasar presupuesto a Administración (Juliana) </t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr">
@@ -3527,12 +3604,12 @@
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Iglesia Impact Valencia</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Administración (Juliana) </t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>Marco Guanuchi</t>
+          <t>Julio Cesar Navia</t>
         </is>
       </c>
       <c r="H33" s="10" t="inlineStr">
@@ -3563,7 +3640,7 @@
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>MÁXIMA URGENCIA — reservar con tiempo</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Buscar alquiler y pasar presupuesto a Administración (Juliana) </t>
         </is>
       </c>
       <c r="G34" s="10" t="inlineStr">
@@ -3599,7 +3676,7 @@
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
-          <t>MÁXIMA URGENCIA</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): MÁXIMA URGENCIA</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
@@ -3635,7 +3712,7 @@
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Valorar opciones con Mateo y Jefferson</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Valorar opciones con Mateo y Jefferson</t>
         </is>
       </c>
       <c r="G36" s="10" t="inlineStr">
@@ -3671,7 +3748,7 @@
       </c>
       <c r="F37" s="9" t="inlineStr">
         <is>
-          <t>Valorar opción con Jefferson</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Valorar opción con Jefferson</t>
         </is>
       </c>
       <c r="G37" s="10" t="inlineStr">
@@ -3707,7 +3784,7 @@
       </c>
       <c r="F38" s="9" t="inlineStr">
         <is>
-          <t>MÁXIMA URGENCIA</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Buscar alquiler y pasar presupuesto a Administración (Juliana) </t>
         </is>
       </c>
       <c r="G38" s="10" t="inlineStr">
@@ -3743,7 +3820,7 @@
       </c>
       <c r="F39" s="9" t="inlineStr">
         <is>
-          <t>MÁXIMA URGENCIA</t>
+          <t xml:space="preserve">CONFIRMADO 17 ago (version final Mariano): Buscar alquiler y pasar presupuesto a Administración (Juliana) </t>
         </is>
       </c>
       <c r="G39" s="10" t="inlineStr">
@@ -3779,7 +3856,7 @@
       </c>
       <c r="F40" s="9" t="inlineStr">
         <is>
-          <t>Hombre del pueblo</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Hombre del pueblo</t>
         </is>
       </c>
       <c r="G40" s="10" t="inlineStr">
@@ -3815,9 +3892,19 @@
           <t>30 sacos</t>
         </is>
       </c>
-      <c r="F41" s="9" t="n"/>
-      <c r="G41" s="10" t="n"/>
-      <c r="H41" s="10" t="n"/>
+      <c r="F41" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA  Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="19">
       <c r="A42" s="7" t="inlineStr">
@@ -3969,7 +4056,7 @@
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>Valorar opción con Richard</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Valorar opción con Richard</t>
         </is>
       </c>
       <c r="G46" s="10" t="inlineStr">
@@ -4067,9 +4154,19 @@
       <c r="E49" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="F49" s="9" t="n"/>
-      <c r="G49" s="10" t="n"/>
-      <c r="H49" s="10" t="n"/>
+      <c r="F49" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA  Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G49" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H49" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="19">
       <c r="A50" s="7" t="inlineStr">
@@ -4091,9 +4188,19 @@
       <c r="E50" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="F50" s="9" t="n"/>
-      <c r="G50" s="10" t="n"/>
-      <c r="H50" s="10" t="n"/>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA</t>
+        </is>
+      </c>
+      <c r="G50" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H50" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="19">
       <c r="A51" s="7" t="inlineStr">
@@ -4115,9 +4222,19 @@
       <c r="E51" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F51" s="9" t="n"/>
-      <c r="G51" s="10" t="n"/>
-      <c r="H51" s="10" t="n"/>
+      <c r="F51" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G51" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H51" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="19">
       <c r="A52" s="7" t="inlineStr">
@@ -4139,9 +4256,19 @@
       <c r="E52" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="F52" s="9" t="n"/>
-      <c r="G52" s="10" t="n"/>
-      <c r="H52" s="10" t="n"/>
+      <c r="F52" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y SEGURIDAD</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H52" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="53" ht="15.75" customHeight="1" s="19">
       <c r="A53" s="7" t="inlineStr">
@@ -4163,9 +4290,19 @@
       <c r="E53" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="F53" s="9" t="n"/>
-      <c r="G53" s="10" t="n"/>
-      <c r="H53" s="10" t="n"/>
+      <c r="F53" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA  Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G53" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H53" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1" s="19">
       <c r="A54" s="7" t="inlineStr">
@@ -4190,8 +4327,16 @@
         <v>100</v>
       </c>
       <c r="F54" s="9" t="n"/>
-      <c r="G54" s="10" t="n"/>
-      <c r="H54" s="10" t="n"/>
+      <c r="G54" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H54" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="15.75" customHeight="1" s="19">
       <c r="A55" s="7" t="inlineStr">
@@ -4218,8 +4363,16 @@
         <v>200</v>
       </c>
       <c r="F55" s="9" t="n"/>
-      <c r="G55" s="10" t="n"/>
-      <c r="H55" s="10" t="n"/>
+      <c r="G55" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H55" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15.75" customHeight="1" s="19">
       <c r="A56" s="7" t="inlineStr">
@@ -4241,9 +4394,19 @@
       <c r="E56" s="9" t="n">
         <v>100</v>
       </c>
-      <c r="F56" s="9" t="n"/>
-      <c r="G56" s="10" t="n"/>
-      <c r="H56" s="10" t="n"/>
+      <c r="F56" s="9" t="inlineStr">
+        <is>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA</t>
+        </is>
+      </c>
+      <c r="G56" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H56" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="57" ht="15.75" customHeight="1" s="19">
       <c r="A57" s="7" t="inlineStr">
@@ -4270,8 +4433,16 @@
         <v>4</v>
       </c>
       <c r="F57" s="9" t="n"/>
-      <c r="G57" s="10" t="n"/>
-      <c r="H57" s="10" t="n"/>
+      <c r="G57" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H57" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15.75" customHeight="1" s="19">
       <c r="A58" s="7" t="inlineStr">
@@ -4298,8 +4469,16 @@
         <v>100</v>
       </c>
       <c r="F58" s="9" t="n"/>
-      <c r="G58" s="10" t="n"/>
-      <c r="H58" s="10" t="n"/>
+      <c r="G58" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H58" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15.75" customHeight="1" s="19">
       <c r="A59" s="7" t="inlineStr">
@@ -4322,8 +4501,16 @@
         <v>100</v>
       </c>
       <c r="F59" s="9" t="n"/>
-      <c r="G59" s="10" t="n"/>
-      <c r="H59" s="10" t="n"/>
+      <c r="G59" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H59" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="15.75" customHeight="1" s="19">
       <c r="A60" s="7" t="inlineStr">
@@ -4346,8 +4533,16 @@
         <v>100</v>
       </c>
       <c r="F60" s="9" t="n"/>
-      <c r="G60" s="10" t="n"/>
-      <c r="H60" s="10" t="n"/>
+      <c r="G60" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H60" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="15.75" customHeight="1" s="19">
       <c r="A61" s="7" t="inlineStr">
@@ -4370,8 +4565,16 @@
         <v>100</v>
       </c>
       <c r="F61" s="9" t="n"/>
-      <c r="G61" s="10" t="n"/>
-      <c r="H61" s="10" t="n"/>
+      <c r="G61" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H61" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="15.75" customHeight="1" s="19">
       <c r="A62" s="7" t="inlineStr">
@@ -4396,8 +4599,16 @@
         <v>100</v>
       </c>
       <c r="F62" s="9" t="n"/>
-      <c r="G62" s="10" t="n"/>
-      <c r="H62" s="10" t="n"/>
+      <c r="G62" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H62" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="15.75" customHeight="1" s="19">
       <c r="A63" s="7" t="inlineStr">
@@ -4424,8 +4635,16 @@
         <v>100</v>
       </c>
       <c r="F63" s="9" t="n"/>
-      <c r="G63" s="10" t="n"/>
-      <c r="H63" s="10" t="n"/>
+      <c r="G63" s="10" t="inlineStr">
+        <is>
+          <t>Marco Guanuchi</t>
+        </is>
+      </c>
+      <c r="H63" s="10" t="inlineStr">
+        <is>
+          <t>9 sept</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="15.75" customHeight="1" s="19">
       <c r="A64" s="13" t="inlineStr">
@@ -4485,7 +4704,7 @@
       </c>
       <c r="F65" s="9" t="inlineStr">
         <is>
-          <t>⚠ Retro decía faltan 2 — confirmar cuál dato es correcto</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): ⚠ Retro decía faltan 2 — confirmar cuál dato es correcto</t>
         </is>
       </c>
       <c r="G65" s="10" t="inlineStr">
@@ -4593,7 +4812,7 @@
       </c>
       <c r="F68" s="9" t="inlineStr">
         <is>
-          <t>Colgar lona piedra Xodos</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Colgar lona piedra Xodos</t>
         </is>
       </c>
       <c r="G68" s="10" t="inlineStr">
@@ -4631,7 +4850,7 @@
       </c>
       <c r="F69" s="9" t="inlineStr">
         <is>
-          <t>Cartel bienvenida</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Cartel bienvenida</t>
         </is>
       </c>
       <c r="G69" s="10" t="inlineStr">
@@ -4829,7 +5048,7 @@
       <c r="E75" s="9" t="n"/>
       <c r="F75" s="9" t="inlineStr">
         <is>
-          <t>Construcción a cargo de Marcos Chiriguaya, confirmar que lo tiene listo</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Construcción a cargo de Marcos Chiriguaya, confirmar que lo tiene listo</t>
         </is>
       </c>
       <c r="G75" s="10" t="inlineStr">
@@ -4867,7 +5086,7 @@
       </c>
       <c r="F76" s="9" t="inlineStr">
         <is>
-          <t>Ya completo — solo confirmar que están en almacén</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Ya completo — solo confirmar que están en almacén</t>
         </is>
       </c>
       <c r="G76" s="10" t="inlineStr">
@@ -5671,7 +5890,7 @@
       </c>
       <c r="F101" s="9" t="inlineStr">
         <is>
-          <t>Marcos Chiriguaya</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Marcos Chiriguaya</t>
         </is>
       </c>
       <c r="G101" s="10" t="inlineStr">
@@ -5707,7 +5926,7 @@
       </c>
       <c r="F102" s="9" t="inlineStr">
         <is>
-          <t>1 Marcos J. + buscar otro</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): 1 Marcos J. + buscar otro</t>
         </is>
       </c>
       <c r="G102" s="10" t="inlineStr">
@@ -5743,7 +5962,7 @@
       </c>
       <c r="F103" s="9" t="inlineStr">
         <is>
-          <t>Marcos Jurado</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Marcos Jurado</t>
         </is>
       </c>
       <c r="G103" s="10" t="inlineStr">
@@ -5779,7 +5998,7 @@
       </c>
       <c r="F104" s="9" t="inlineStr">
         <is>
-          <t>Marcos Chiriguaya</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Marcos Chiriguaya</t>
         </is>
       </c>
       <c r="G104" s="10" t="inlineStr">
@@ -5815,7 +6034,7 @@
       </c>
       <c r="F105" s="9" t="inlineStr">
         <is>
-          <t>Iglesia Impact Valencia</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): Iglesia Impact Valencia</t>
         </is>
       </c>
       <c r="G105" s="10" t="inlineStr">
@@ -6037,7 +6256,7 @@
       </c>
       <c r="H111" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6071,7 +6290,7 @@
       </c>
       <c r="H112" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6105,7 +6324,7 @@
       </c>
       <c r="H113" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6358,7 @@
       </c>
       <c r="H114" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6173,7 +6392,7 @@
       </c>
       <c r="H115" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6426,7 @@
       </c>
       <c r="H116" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6460,7 @@
       </c>
       <c r="H117" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6275,7 +6494,7 @@
       </c>
       <c r="H118" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6309,7 +6528,7 @@
       </c>
       <c r="H119" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6345,7 +6564,7 @@
       </c>
       <c r="H120" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6379,7 +6598,7 @@
       </c>
       <c r="H121" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6415,7 +6634,7 @@
       </c>
       <c r="H122" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6668,7 @@
       </c>
       <c r="H123" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6485,7 +6704,7 @@
       </c>
       <c r="H124" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6521,7 +6740,7 @@
       </c>
       <c r="H125" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6555,7 +6774,7 @@
       </c>
       <c r="H126" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6810,7 @@
       </c>
       <c r="H127" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6627,7 +6846,7 @@
       </c>
       <c r="H128" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6663,7 +6882,7 @@
       </c>
       <c r="H129" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6918,7 @@
       </c>
       <c r="H130" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6735,7 +6954,7 @@
       </c>
       <c r="H131" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6771,7 +6990,7 @@
       </c>
       <c r="H132" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6807,7 +7026,7 @@
       </c>
       <c r="H133" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6841,7 +7060,7 @@
       </c>
       <c r="H134" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6875,7 +7094,7 @@
       </c>
       <c r="H135" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6909,7 +7128,7 @@
       </c>
       <c r="H136" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6943,7 +7162,7 @@
       </c>
       <c r="H137" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -6979,7 +7198,7 @@
       </c>
       <c r="H138" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7015,7 +7234,7 @@
       </c>
       <c r="H139" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7051,7 +7270,7 @@
       </c>
       <c r="H140" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7304,7 @@
       </c>
       <c r="H141" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7121,7 +7340,7 @@
       </c>
       <c r="H142" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7155,7 +7374,7 @@
       </c>
       <c r="H143" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7191,7 +7410,7 @@
       </c>
       <c r="H144" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7227,7 +7446,7 @@
       </c>
       <c r="H145" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7263,7 +7482,7 @@
       </c>
       <c r="H146" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7299,7 +7518,7 @@
       </c>
       <c r="H147" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7333,7 +7552,7 @@
       </c>
       <c r="H148" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7367,7 +7586,7 @@
       </c>
       <c r="H149" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7620,7 @@
       </c>
       <c r="H150" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7437,7 +7656,7 @@
       </c>
       <c r="H151" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7473,7 +7692,7 @@
       </c>
       <c r="H152" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7505,7 +7724,7 @@
       </c>
       <c r="H153" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7541,7 +7760,7 @@
       </c>
       <c r="H154" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7577,7 +7796,7 @@
       </c>
       <c r="H155" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7613,7 +7832,7 @@
       </c>
       <c r="H156" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7649,7 +7868,7 @@
       </c>
       <c r="H157" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7683,7 +7902,7 @@
       </c>
       <c r="H158" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7717,7 +7936,7 @@
       </c>
       <c r="H159" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7751,7 +7970,7 @@
       </c>
       <c r="H160" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7785,7 +8004,7 @@
       </c>
       <c r="H161" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7821,7 +8040,7 @@
       </c>
       <c r="H162" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7857,7 +8076,7 @@
       </c>
       <c r="H163" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7893,7 +8112,7 @@
       </c>
       <c r="H164" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7929,7 +8148,7 @@
       </c>
       <c r="H165" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -7965,7 +8184,7 @@
       </c>
       <c r="H166" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -8001,7 +8220,7 @@
       </c>
       <c r="H167" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -8035,7 +8254,7 @@
       </c>
       <c r="H168" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -8069,7 +8288,7 @@
       </c>
       <c r="H169" s="10" t="inlineStr">
         <is>
-          <t>28 sept</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -8131,7 +8350,7 @@
       <c r="E171" s="9" t="n"/>
       <c r="F171" s="9" t="inlineStr">
         <is>
-          <t>O coordinar hacerlo días antes; David puede prestar herramienta de obra</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): O coordinar hacerlo días antes; David puede prestar herramienta de obra</t>
         </is>
       </c>
       <c r="G171" s="10" t="inlineStr">
@@ -8141,7 +8360,7 @@
       </c>
       <c r="H171" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -8171,7 +8390,7 @@
       </c>
       <c r="H172" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -8201,7 +8420,7 @@
       </c>
       <c r="H173" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>26 ago</t>
         </is>
       </c>
     </row>
@@ -8225,7 +8444,7 @@
       <c r="E174" s="9" t="n"/>
       <c r="F174" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta.</t>
         </is>
       </c>
       <c r="G174" s="10" t="inlineStr">
@@ -8259,7 +8478,7 @@
       <c r="E175" s="9" t="n"/>
       <c r="F175" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta.</t>
         </is>
       </c>
       <c r="G175" s="10" t="inlineStr">
@@ -8293,7 +8512,7 @@
       <c r="E176" s="9" t="n"/>
       <c r="F176" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta.</t>
         </is>
       </c>
       <c r="G176" s="10" t="inlineStr">
@@ -8327,7 +8546,7 @@
       <c r="E177" s="9" t="n"/>
       <c r="F177" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta.</t>
         </is>
       </c>
       <c r="G177" s="10" t="inlineStr">
@@ -8361,7 +8580,7 @@
       <c r="E178" s="9" t="n"/>
       <c r="F178" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta.</t>
         </is>
       </c>
       <c r="G178" s="10" t="inlineStr">
@@ -8395,7 +8614,7 @@
       <c r="E179" s="9" t="n"/>
       <c r="F179" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta.</t>
         </is>
       </c>
       <c r="G179" s="10" t="inlineStr">
@@ -8429,7 +8648,7 @@
       <c r="E180" s="9" t="n"/>
       <c r="F180" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
+          <t>CONFIRMADO 17 ago (version final Mariano): ALMACEN RUGE (ya en stock) — confirmar con Adrián Rivera que esté en buen estado y la cantidad correcta.</t>
         </is>
       </c>
       <c r="G180" s="10" t="inlineStr">
@@ -8463,11 +8682,17 @@
       <c r="E181" s="9" t="n"/>
       <c r="F181" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G181" s="10" t="n"/>
-      <c r="H181" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G181" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H181" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="182" ht="15.75" customHeight="1" s="19">
       <c r="A182" s="7" t="inlineStr">
@@ -8489,11 +8714,17 @@
       <c r="E182" s="9" t="n"/>
       <c r="F182" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G182" s="10" t="n"/>
-      <c r="H182" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G182" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H182" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="183" ht="15.75" customHeight="1" s="19">
       <c r="A183" s="7" t="inlineStr">
@@ -8515,11 +8746,17 @@
       <c r="E183" s="9" t="n"/>
       <c r="F183" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G183" s="10" t="n"/>
-      <c r="H183" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G183" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H183" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="184" ht="15.75" customHeight="1" s="19">
       <c r="A184" s="7" t="inlineStr">
@@ -8541,11 +8778,17 @@
       <c r="E184" s="9" t="n"/>
       <c r="F184" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G184" s="10" t="n"/>
-      <c r="H184" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G184" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H184" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="185" ht="15.75" customHeight="1" s="19">
       <c r="A185" s="7" t="inlineStr">
@@ -8567,11 +8810,17 @@
       <c r="E185" s="9" t="n"/>
       <c r="F185" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G185" s="10" t="n"/>
-      <c r="H185" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G185" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H185" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="186" ht="15.75" customHeight="1" s="19">
       <c r="A186" s="7" t="inlineStr">
@@ -8593,11 +8842,17 @@
       <c r="E186" s="9" t="n"/>
       <c r="F186" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G186" s="10" t="n"/>
-      <c r="H186" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y GUIAS</t>
+        </is>
+      </c>
+      <c r="G186" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H186" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="187" ht="15.75" customHeight="1" s="19">
       <c r="A187" s="7" t="inlineStr">
@@ -8619,11 +8874,17 @@
       <c r="E187" s="9" t="n"/>
       <c r="F187" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G187" s="10" t="n"/>
-      <c r="H187" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G187" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H187" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="188" ht="15.75" customHeight="1" s="19">
       <c r="A188" s="7" t="inlineStr">
@@ -8645,11 +8906,17 @@
       <c r="E188" s="9" t="n"/>
       <c r="F188" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G188" s="10" t="n"/>
-      <c r="H188" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G188" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H188" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="189" ht="15.75" customHeight="1" s="19">
       <c r="A189" s="7" t="inlineStr">
@@ -8671,11 +8938,17 @@
       <c r="E189" s="9" t="n"/>
       <c r="F189" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G189" s="10" t="n"/>
-      <c r="H189" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G189" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H189" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="190" ht="15.75" customHeight="1" s="19">
       <c r="A190" s="7" t="inlineStr">
@@ -8697,11 +8970,17 @@
       <c r="E190" s="9" t="n"/>
       <c r="F190" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G190" s="10" t="n"/>
-      <c r="H190" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y GUIAS</t>
+        </is>
+      </c>
+      <c r="G190" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H190" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="191" ht="15.75" customHeight="1" s="19">
       <c r="A191" s="7" t="inlineStr">
@@ -8723,11 +9002,17 @@
       <c r="E191" s="9" t="n"/>
       <c r="F191" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G191" s="10" t="n"/>
-      <c r="H191" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G191" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H191" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="192" ht="15.75" customHeight="1" s="19">
       <c r="A192" s="7" t="inlineStr">
@@ -8749,11 +9034,17 @@
       <c r="E192" s="9" t="n"/>
       <c r="F192" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G192" s="10" t="n"/>
-      <c r="H192" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G192" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H192" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="193" ht="15.75" customHeight="1" s="19">
       <c r="A193" s="7" t="inlineStr">
@@ -8775,11 +9066,17 @@
       <c r="E193" s="9" t="n"/>
       <c r="F193" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G193" s="10" t="n"/>
-      <c r="H193" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G193" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H193" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="194" ht="15.75" customHeight="1" s="19">
       <c r="A194" s="7" t="inlineStr">
@@ -8801,11 +9098,17 @@
       <c r="E194" s="9" t="n"/>
       <c r="F194" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G194" s="10" t="n"/>
-      <c r="H194" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y SEGURIDAD</t>
+        </is>
+      </c>
+      <c r="G194" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H194" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="195" ht="15.75" customHeight="1" s="19">
       <c r="A195" s="7" t="inlineStr">
@@ -8827,11 +9130,17 @@
       <c r="E195" s="9" t="n"/>
       <c r="F195" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G195" s="10" t="n"/>
-      <c r="H195" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G195" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H195" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="196" ht="15.75" customHeight="1" s="19">
       <c r="A196" s="7" t="inlineStr">
@@ -8853,11 +9162,17 @@
       <c r="E196" s="9" t="n"/>
       <c r="F196" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G196" s="10" t="n"/>
-      <c r="H196" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G196" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H196" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="197" ht="15.75" customHeight="1" s="19">
       <c r="A197" s="7" t="inlineStr">
@@ -8879,11 +9194,17 @@
       <c r="E197" s="9" t="n"/>
       <c r="F197" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G197" s="10" t="n"/>
-      <c r="H197" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G197" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H197" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="198" ht="15.75" customHeight="1" s="19">
       <c r="A198" s="7" t="inlineStr">
@@ -8905,11 +9226,17 @@
       <c r="E198" s="9" t="n"/>
       <c r="F198" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G198" s="10" t="n"/>
-      <c r="H198" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G198" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H198" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="199" ht="15.75" customHeight="1" s="19">
       <c r="A199" s="7" t="inlineStr">
@@ -8931,11 +9258,17 @@
       <c r="E199" s="9" t="n"/>
       <c r="F199" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G199" s="10" t="n"/>
-      <c r="H199" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G199" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H199" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="200" ht="15.75" customHeight="1" s="19">
       <c r="A200" s="7" t="inlineStr">
@@ -8957,11 +9290,17 @@
       <c r="E200" s="9" t="n"/>
       <c r="F200" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G200" s="10" t="n"/>
-      <c r="H200" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G200" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H200" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="201" ht="15.75" customHeight="1" s="19">
       <c r="A201" s="7" t="inlineStr">
@@ -8983,11 +9322,17 @@
       <c r="E201" s="9" t="n"/>
       <c r="F201" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G201" s="10" t="n"/>
-      <c r="H201" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y SEGURIDAD</t>
+        </is>
+      </c>
+      <c r="G201" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H201" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="202" ht="15.75" customHeight="1" s="19">
       <c r="A202" s="7" t="inlineStr">
@@ -9009,11 +9354,17 @@
       <c r="E202" s="9" t="n"/>
       <c r="F202" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G202" s="10" t="n"/>
-      <c r="H202" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G202" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H202" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="203" ht="15.75" customHeight="1" s="19">
       <c r="A203" s="7" t="inlineStr">
@@ -9035,11 +9386,17 @@
       <c r="E203" s="9" t="n"/>
       <c r="F203" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G203" s="10" t="n"/>
-      <c r="H203" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G203" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H203" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="204" ht="15.75" customHeight="1" s="19">
       <c r="A204" s="7" t="inlineStr">
@@ -9061,11 +9418,17 @@
       <c r="E204" s="9" t="n"/>
       <c r="F204" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G204" s="10" t="n"/>
-      <c r="H204" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y GUIAS</t>
+        </is>
+      </c>
+      <c r="G204" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H204" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="205" ht="15.75" customHeight="1" s="19">
       <c r="A205" s="7" t="inlineStr">
@@ -9087,11 +9450,17 @@
       <c r="E205" s="9" t="n"/>
       <c r="F205" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G205" s="10" t="n"/>
-      <c r="H205" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G205" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H205" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="206" ht="15.75" customHeight="1" s="19">
       <c r="A206" s="7" t="inlineStr">
@@ -9113,11 +9482,17 @@
       <c r="E206" s="9" t="n"/>
       <c r="F206" s="9" t="inlineStr">
         <is>
-          <t>ALMACEN RUGE (ya en stock) — no se discutió en la llamada del 17 ago, pendiente asignar encargado y verificar en la reunión del miércoles. Agregado 17 ago al detectar que faltaba en el detalle original.</t>
-        </is>
-      </c>
-      <c r="G206" s="10" t="n"/>
-      <c r="H206" s="10" t="n"/>
+          <t>CONFIRMADO 17 ago (version final Mariano): LOGÍSTICA Y EVENTOS</t>
+        </is>
+      </c>
+      <c r="G206" s="10" t="inlineStr">
+        <is>
+          <t>David Luzuriaga</t>
+        </is>
+      </c>
+      <c r="H206" s="27" t="n">
+        <v>46267</v>
+      </c>
     </row>
     <row r="207" ht="15.75" customHeight="1" s="19"/>
     <row r="208" ht="15.75" customHeight="1" s="19"/>

</xml_diff>